<commit_message>
now added new feature
</commit_message>
<xml_diff>
--- a/teacher_details.xlsx
+++ b/teacher_details.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2550,6 +2550,50 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>66e99fdf34b6696aecdbe4bb</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>TulikaJha Ma'am</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>9953339722</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5eb393ee95fab7468a79d189/ADMIN/cb402c28-09ed-4ceb-93d0-eeff3a73331c.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>614f5a4a7517d40019933849</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>YogeshJain Sir</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>8118855459</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://static.pw.live/5eb393ee95fab7468a79d189/ADMIN/b749edd6-cbdc-4564-ab7c-7101fc08ca1e.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>